<commit_message>
Make the PL28 and coach formats as similar as possible
Approved format change (VERSIONS.md, 2026-10-26):
- Same reading rules: sheet names and headers ignore capitals, lowercase
  day letters, alphabetical days, blank rows in overall skipped and two in
  a row end it, block rows need only a name or a variant.
- One overall layout for both: week | giorno (dates) | tipo | lifts, read
  by parse-common.js scanOverall(). PL28 gains dates and tipo; its old
  week | fase layout is still read.
- PL28 accessori: Rep and Intensità accept load formulas and placeholders.
- Exports and templates write the shared layout, formatVersion 2.
- tests/formats.test.js covers every new rule; all fixtures unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/PL-template-PL28.xlsx
+++ b/examples/PL-template-PL28.xlsx
@@ -20,14 +20,28 @@
     <author>Author</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t>Riga con A vuota = nuovo blocco: nome in B, varianti sotto le alzate.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Riga con A vuota = nuovo blocco (nome in B, varianti a destra). Tipo di settimana: normale (o vuoto), scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara</t>
+          <t>Date della settimana (testo libero, facoltativo).</t>
         </r>
       </text>
     </comment>
     <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <t>Tipo di settimana: normale (o vuoto), scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <t>Carico dai massimali: ="4x5 "&amp;MROUND(Massimali!$B$3*0.57,2.5)&amp;"kg" (riga 3 = prima alzata, 0.57 = 57%, arrotondato a 2,5), oppure testo con segnaposto: 4x5 {Squat .57}kg</t>
@@ -44,6 +58,13 @@
     <author>Author</author>
   </authors>
   <commentList>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Rep e Intensità possono contenere carichi. Carico dai massimali: ="4x5 "&amp;MROUND(Massimali!$B$3*0.57,2.5)&amp;"kg" (riga 3 = prima alzata, 0.57 = 57%, arrotondato a 2,5), oppure testo con segnaposto: 4x5 {Squat .57}kg</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G1" authorId="0">
       <text>
         <r>
@@ -56,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>Template PL – formato PL28 (accessori uguali per tutto il blocco)</t>
   </si>
@@ -70,10 +91,13 @@
     <t>• Massimali: nome in colonna A, massimale in colonna B, dalla riga 3. Le formule puntano alla riga: Massimali!$B$3 = prima alzata.</t>
   </si>
   <si>
-    <t>• overall, riga 1: week | fase | una colonna per alzata "Nome (giorno)", es. "Squat (A)".</t>
-  </si>
-  <si>
-    <t>• overall, riga di blocco: A vuota, nome del blocco in B, varianti sotto ogni alzata. Righe di settimana: numero in A (1, 2, 3… senza buchi), tipo in B, prescrizioni.</t>
+    <t>• overall, riga 1: week | giorno | tipo | una colonna per alzata "Nome (giorno)", es. "Squat (A)". Le colonne vuote fanno da separatore.</t>
+  </si>
+  <si>
+    <t>• overall, riga di blocco: A vuota, nome del blocco in B, varianti sotto ogni alzata. Righe di settimana: numero in A (1, 2, 3… senza buchi), date in B (facoltative), tipo in C, prescrizioni.</t>
+  </si>
+  <si>
+    <t>• Righe vuote tra i blocchi vanno bene; due righe vuote di fila chiudono il foglio.</t>
   </si>
   <si>
     <t>• Tipo di settimana (menu a tendina): normale (o vuoto), scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara.</t>
@@ -82,7 +106,7 @@
     <t>• Prescrizioni: testo libero; carichi con la formula ="4x5 "&amp;MROUND(Massimali!$B$3*0.75,2.5)&amp;"kg" oppure col segnaposto 4x5 {Squat .75}kg. Cella vuota = alzata non fatta quella settimana.</t>
   </si>
   <si>
-    <t>• accessori: Giorno | Esercizio | Istruzioni | Gruppo | Rep | Intensità, poi una colonna "Serie B…" per blocco (intero, 0 = non fatto).</t>
+    <t>• accessori: Giorno | Esercizio | Istruzioni | Gruppo | Rep | Intensità, poi una colonna "Serie B…" per blocco (intero, 0 = non fatto). Rep e Intensità possono contenere carichi, come le prescrizioni.</t>
   </si>
   <si>
     <t>• Nelle settimane transizione, scarico e test l'app toglie 1 serie agli accessori e aggiunge 1 al RIR.</t>
@@ -109,7 +133,10 @@
     <t>week</t>
   </si>
   <si>
-    <t>fase</t>
+    <t>giorno</t>
+  </si>
+  <si>
+    <t>tipo</t>
   </si>
   <si>
     <t>Squat (A)</t>
@@ -599,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -658,6 +685,11 @@
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -677,12 +709,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2">
         <v>180</v>
@@ -690,7 +722,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2">
         <v>120</v>
@@ -698,7 +730,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2">
         <v>210</v>
@@ -706,7 +738,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <f>SUM(B3:B5)</f>
@@ -721,76 +753,82 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="6" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>23</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="str">
         <f>"4x5 "&amp;MROUND(Massimali!$B$3*0.75,2.5)&amp;"kg"</f>
         <v>4x5 135kg</v>
       </c>
-      <c r="D3" s="2" t="str">
+      <c r="E3" s="2" t="str">
         <f>"5x5 "&amp;MROUND(Massimali!$B$4*0.72,2.5)&amp;"kg"</f>
         <v>5x5 87,5kg</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="str">
         <f>MROUND(Massimali!$B$4*0.65,2.5)&amp;"kg 30-35RT"</f>
         <v>77,5kg 30-35RT</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorStyle="stop" errorTitle="Valore non ammesso" error="Usa uno di: normale, scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara" sqref="B2:B400">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valore non ammesso" error="Usa uno di: normale, scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara" sqref="C2:C400">
       <formula1>"normale,scarico,transizione,ramping,intensificazione,picco,taper,entrata,test,gara"</formula1>
     </dataValidation>
   </dataValidations>
@@ -816,45 +854,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G2" s="2">
         <v>3</v>
@@ -862,20 +900,20 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G3" s="2">
         <v>3</v>
@@ -883,20 +921,20 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4" s="2">
         <v>3</v>
@@ -925,10 +963,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lift types in overall, and lift columns grouped by lift
Approved format change (VERSIONS.md, 2026-10-26):
- Optional row 2 in overall: A2 = "tipo alzata", free text under each
  lift column (stressante, rigenerante...). Stored as liftType on items
  (schema 3; migrate() adds null), shown as a tag next to the lift name.
  Coach format: a log row takes the type of the overall column its E
  points at.
- Exports and templates write the tipo alzata row and group lift columns
  by lift (Massimali order, others last), then by day. PL28 exports fall
  back to day grouping when lift grouping would reorder a day's lifts.
- tests/lift-types.test.js; docs updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/PL-template-PL28.xlsx
+++ b/examples/PL-template-PL28.xlsx
@@ -48,6 +48,13 @@
         </r>
       </text>
     </comment>
+    <comment ref="A2" authorId="0">
+      <text>
+        <r>
+          <t>Tipo di ogni alzata (facoltativo, testo libero): stressante, rigenerante, tecnica… L'app lo mostra accanto al nome.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -77,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>Template PL – formato PL28 (accessori uguali per tutto il blocco)</t>
   </si>
@@ -91,7 +98,10 @@
     <t>• Massimali: nome in colonna A, massimale in colonna B, dalla riga 3. Le formule puntano alla riga: Massimali!$B$3 = prima alzata.</t>
   </si>
   <si>
-    <t>• overall, riga 1: week | giorno | tipo | una colonna per alzata "Nome (giorno)", es. "Squat (A)". Le colonne vuote fanno da separatore.</t>
+    <t>• overall, riga 1: week | giorno | tipo | una colonna per alzata "Nome (giorno)", es. "Squat (A)", raggruppate per alzata (Squat A, Squat C… poi Panca). Le colonne vuote fanno da separatore.</t>
+  </si>
+  <si>
+    <t>• overall, riga 2 (facoltativa): "tipo alzata" in A e sotto ogni alzata il suo tipo (stressante, rigenerante, tecnica…, testo libero). L'app lo mostra accanto al nome.</t>
   </si>
   <si>
     <t>• overall, riga di blocco: A vuota, nome del blocco in B, varianti sotto ogni alzata. Righe di settimana: numero in A (1, 2, 3… senza buchi), date in B (facoltative), tipo in C, prescrizioni.</t>
@@ -145,10 +155,19 @@
     <t>Panca (A)</t>
   </si>
   <si>
+    <t>Panca var. (C)</t>
+  </si>
+  <si>
     <t>Stacco (B)</t>
   </si>
   <si>
-    <t>Panca var. (C)</t>
+    <t>tipo alzata</t>
+  </si>
+  <si>
+    <t>stressante</t>
+  </si>
+  <si>
+    <t>rigenerante</t>
   </si>
   <si>
     <t>Blocco 1 – ESEMPIO</t>
@@ -626,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -690,6 +709,11 @@
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -709,12 +733,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2">
         <v>180</v>
@@ -722,7 +746,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2">
         <v>120</v>
@@ -730,7 +754,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2">
         <v>210</v>
@@ -738,7 +762,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <f>SUM(B3:B5)</f>
@@ -753,10 +777,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="7" width="24" customWidth="1"/>
@@ -764,72 +788,94 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="A2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2" t="str">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="str">
         <f>"4x5 "&amp;MROUND(Massimali!$B$3*0.75,2.5)&amp;"kg"</f>
         <v>4x5 135kg</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E4" s="2" t="str">
         <f>"5x5 "&amp;MROUND(Massimali!$B$4*0.72,2.5)&amp;"kg"</f>
         <v>5x5 87,5kg</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="2" t="str">
+      <c r="F4" s="2" t="str">
         <f>MROUND(Massimali!$B$4*0.65,2.5)&amp;"kg 30-35RT"</f>
         <v>77,5kg 30-35RT</v>
       </c>
+      <c r="G4" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valore non ammesso" error="Usa uno di: normale, scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara" sqref="C2:C400">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valore non ammesso" error="Usa uno di: normale, scarico, transizione, ramping, intensificazione, picco, taper, entrata, test, gara" sqref="C3:C400">
       <formula1>"normale,scarico,transizione,ramping,intensificazione,picco,taper,entrata,test,gara"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" errorStyle="stop" errorTitle="Valore non ammesso" error="Usa uno di: stressante, rigenerante, tecnica, stimolo, volume" sqref="D2:G2">
+      <formula1>"stressante,rigenerante,tecnica,stimolo,volume"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -854,45 +900,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G2" s="2">
         <v>3</v>
@@ -900,20 +946,20 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G3" s="2">
         <v>3</v>
@@ -921,20 +967,20 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G4" s="2">
         <v>3</v>
@@ -963,7 +1009,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B1">
         <v>2</v>

</xml_diff>